<commit_message>
Add article-list block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (16):
- blocks/article-list/article-list.css
- blocks/article-list/article-list.js
- docs/query-index-config.md
- helix-query.yaml
- tools/importer/import-blog.bundle.js
- tools/importer/import-blog.js
- tools/importer/reports/blog/ace-pro-court-polo.report.json
- tools/importer/reports/blog/fashion-blog-post.report.json
- tools/importer/reports/blog/fashion-trends-young-culture.report.json
- tools/importer/reports/blog/fashion-trends-young-style.report.json
- tools/importer/reports/blog/flip-flop-summer-style.report.json
- tools/importer/reports/blog/latest-trends-young-casual-fashion.report.json
- tools/importer/reports/blog/street-style-trends.report.json
- tools/importer/reports/import-blog.report.xlsx
- tools/importer/transformers/wknd-trendsetters-blog-metadata.js
- tools/importer/urls-blog.txt
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-blog.report.xlsx
+++ b/tools/importer/reports/import-blog.report.xlsx
@@ -70,7 +70,7 @@
     <t>blog</t>
   </si>
   <si>
-    <t>2026-09-02T06:05:47.696Z</t>
+    <t>2026-09-02T08:46:03.477Z</t>
   </si>
   <si>
     <t>Court cool, street ready — the Ace Pro polo | Fashion Blog</t>
@@ -85,7 +85,7 @@
     <t>blog/fashion-blog-post</t>
   </si>
   <si>
-    <t>2026-09-02T06:07:05.534Z</t>
+    <t>2026-09-02T08:46:28.083Z</t>
   </si>
   <si>
     <t>Game on, style up | Fashion Blog</t>
@@ -100,7 +100,7 @@
     <t>blog/fashion-trends-young-culture</t>
   </si>
   <si>
-    <t>2026-09-02T06:06:56.170Z</t>
+    <t>2026-09-02T08:46:18.884Z</t>
   </si>
   <si>
     <t>Sunkissed and effortless | Fashion Blog</t>
@@ -115,7 +115,7 @@
     <t>blog/fashion-trends-young-style</t>
   </si>
   <si>
-    <t>2026-09-02T06:07:00.852Z</t>
+    <t>2026-09-02T08:46:23.899Z</t>
   </si>
   <si>
     <t>Party fits that pop | Fashion Blog</t>
@@ -130,7 +130,7 @@
     <t>blog/flip-flop-summer-style</t>
   </si>
   <si>
-    <t>2026-09-02T06:06:44.517Z</t>
+    <t>2026-09-02T08:46:08.076Z</t>
   </si>
   <si>
     <t>Slide into summer — flip flops that serve | Fashion Blog</t>
@@ -145,7 +145,7 @@
     <t>blog/latest-trends-young-casual-fashion</t>
   </si>
   <si>
-    <t>2026-09-02T06:06:49.949Z</t>
+    <t>2026-09-02T08:46:14.513Z</t>
   </si>
   <si>
     <t>Tennis style, redefined | Fashion Blog</t>
@@ -160,7 +160,7 @@
     <t>blog/street-style-trends</t>
   </si>
   <si>
-    <t>2026-09-02T06:07:11.434Z</t>
+    <t>2026-09-02T08:46:32.855Z</t>
   </si>
   <si>
     <t>Street style, your way | Fashion Blog</t>

</xml_diff>